<commit_message>
Add functionality to skip entries that are a request to update service list
</commit_message>
<xml_diff>
--- a/data/dockets_input.xlsx
+++ b/data/dockets_input.xlsx
@@ -6,10 +6,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="dockets" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -47,9 +47,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -394,10 +393,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="10.08984375" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
+    <col width="10.08984375" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -415,20 +414,870 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EL25-49</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
+          <t>AD16-16</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>46109</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>AD21-15</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AD22-13</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AD22-5</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AD22-8</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AD23-10</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AD24-11</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>AD24-7</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B9" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AD24-9</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AD25-7</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EC18-137</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EL21-3</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EL21-6</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EL21-94</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EL22-22</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EL22-42</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EL23-16</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>EL23-62</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EL24-80</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EL24-81</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EL24-82</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>EL24-83</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EL24-95</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>EL25-117</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>EL25-43</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EL25-44</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EL25-49</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>EL25-80</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ER18-2123</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ER18-2124</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ER20-2054</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ER21-1111</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ER22-1290</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ER22-2357</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ER22-2467</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ER22-2468</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ER22-2886</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ER22-983</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ER24-115</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ER24-1177</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ER24-1245</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ER24-1290</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ER24-1710</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ER24-1978</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ER24-2007</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ER24-2009</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ER24-2584</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ER24-275</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ER24-2795</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ER24-2796</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ER24-2939</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ER24-3071</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ER24-3154</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ER24-324</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ER24-339</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ER24-401</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ER24-420</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ER24-476</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ER25-1324</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ER25-1445</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ER25-1703</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ER25-1799</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ER25-2500</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ER25-410</t>
+        </is>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ER25-747</t>
+        </is>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ER25-830</t>
+        </is>
+      </c>
+      <c r="B67" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ER25-866</t>
+        </is>
+      </c>
+      <c r="B68" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ER26-925</t>
+        </is>
+      </c>
+      <c r="B69" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>RD22-4</t>
+        </is>
+      </c>
+      <c r="B70" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>RD24-5</t>
+        </is>
+      </c>
+      <c r="B71" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>RD25-1</t>
+        </is>
+      </c>
+      <c r="B72" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>RD25-2</t>
+        </is>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>RD25-3</t>
+        </is>
+      </c>
+      <c r="B74" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>RD26-1</t>
+        </is>
+      </c>
+      <c r="B75" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>RD26-2</t>
+        </is>
+      </c>
+      <c r="B76" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>RD26-3</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>RM18-9</t>
+        </is>
+      </c>
+      <c r="B78" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>RM20-16</t>
+        </is>
+      </c>
+      <c r="B79" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>RM21-17</t>
+        </is>
+      </c>
+      <c r="B80" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>RM22-10</t>
+        </is>
+      </c>
+      <c r="B81" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>RM22-2</t>
+        </is>
+      </c>
+      <c r="B82" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>RM22-7</t>
+        </is>
+      </c>
+      <c r="B83" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>RM24-4</t>
+        </is>
+      </c>
+      <c r="B84" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>RM24-6</t>
+        </is>
+      </c>
+      <c r="B85" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>RM25-3</t>
+        </is>
+      </c>
+      <c r="B86" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>RM26-4</t>
+        </is>
+      </c>
+      <c r="B87" s="1" t="n">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>RR24-2</t>
+        </is>
+      </c>
+      <c r="B88" s="1" t="n">
         <v>46109</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add api module for Illinois Commerce Commission, enable scaling for input/output data files and utilities
</commit_message>
<xml_diff>
--- a/data/dockets_input.xlsx
+++ b/data/dockets_input.xlsx
@@ -6,10 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="dockets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ferc" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="illinois" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -418,7 +419,7 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="3">
@@ -428,7 +429,7 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="4">
@@ -438,7 +439,7 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="5">
@@ -448,7 +449,7 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="6">
@@ -458,7 +459,7 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="7">
@@ -468,7 +469,7 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="8">
@@ -478,7 +479,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="9">
@@ -488,7 +489,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="10">
@@ -498,7 +499,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="11">
@@ -508,7 +509,7 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="12">
@@ -518,7 +519,7 @@
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +529,7 @@
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="14">
@@ -538,7 +539,7 @@
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="15">
@@ -548,7 +549,7 @@
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="16">
@@ -558,7 +559,7 @@
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="17">
@@ -568,7 +569,7 @@
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="18">
@@ -578,7 +579,7 @@
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="19">
@@ -588,7 +589,7 @@
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="20">
@@ -598,7 +599,7 @@
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="21">
@@ -608,7 +609,7 @@
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="22">
@@ -618,7 +619,7 @@
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="23">
@@ -628,7 +629,7 @@
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="24">
@@ -638,7 +639,7 @@
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="25">
@@ -648,7 +649,7 @@
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="26">
@@ -658,7 +659,7 @@
         </is>
       </c>
       <c r="B26" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="27">
@@ -668,7 +669,7 @@
         </is>
       </c>
       <c r="B27" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="28">
@@ -678,7 +679,7 @@
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="29">
@@ -688,7 +689,7 @@
         </is>
       </c>
       <c r="B29" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="30">
@@ -698,7 +699,7 @@
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="31">
@@ -708,7 +709,7 @@
         </is>
       </c>
       <c r="B31" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="32">
@@ -718,7 +719,7 @@
         </is>
       </c>
       <c r="B32" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="33">
@@ -728,7 +729,7 @@
         </is>
       </c>
       <c r="B33" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="34">
@@ -738,7 +739,7 @@
         </is>
       </c>
       <c r="B34" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="35">
@@ -748,7 +749,7 @@
         </is>
       </c>
       <c r="B35" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="36">
@@ -758,7 +759,7 @@
         </is>
       </c>
       <c r="B36" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="37">
@@ -768,7 +769,7 @@
         </is>
       </c>
       <c r="B37" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="38">
@@ -778,7 +779,7 @@
         </is>
       </c>
       <c r="B38" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="39">
@@ -788,7 +789,7 @@
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="40">
@@ -798,7 +799,7 @@
         </is>
       </c>
       <c r="B40" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="41">
@@ -808,7 +809,7 @@
         </is>
       </c>
       <c r="B41" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="42">
@@ -818,7 +819,7 @@
         </is>
       </c>
       <c r="B42" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="43">
@@ -828,7 +829,7 @@
         </is>
       </c>
       <c r="B43" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="44">
@@ -838,7 +839,7 @@
         </is>
       </c>
       <c r="B44" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="45">
@@ -848,7 +849,7 @@
         </is>
       </c>
       <c r="B45" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="46">
@@ -858,7 +859,7 @@
         </is>
       </c>
       <c r="B46" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="47">
@@ -868,7 +869,7 @@
         </is>
       </c>
       <c r="B47" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="48">
@@ -878,7 +879,7 @@
         </is>
       </c>
       <c r="B48" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="49">
@@ -888,7 +889,7 @@
         </is>
       </c>
       <c r="B49" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="50">
@@ -898,7 +899,7 @@
         </is>
       </c>
       <c r="B50" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="51">
@@ -908,7 +909,7 @@
         </is>
       </c>
       <c r="B51" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="52">
@@ -918,7 +919,7 @@
         </is>
       </c>
       <c r="B52" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="53">
@@ -928,7 +929,7 @@
         </is>
       </c>
       <c r="B53" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="54">
@@ -938,7 +939,7 @@
         </is>
       </c>
       <c r="B54" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="55">
@@ -948,7 +949,7 @@
         </is>
       </c>
       <c r="B55" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="56">
@@ -958,7 +959,7 @@
         </is>
       </c>
       <c r="B56" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="57">
@@ -968,7 +969,7 @@
         </is>
       </c>
       <c r="B57" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="58">
@@ -978,7 +979,7 @@
         </is>
       </c>
       <c r="B58" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="59">
@@ -988,7 +989,7 @@
         </is>
       </c>
       <c r="B59" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="60">
@@ -998,7 +999,7 @@
         </is>
       </c>
       <c r="B60" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="61">
@@ -1008,7 +1009,7 @@
         </is>
       </c>
       <c r="B61" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="62">
@@ -1018,7 +1019,7 @@
         </is>
       </c>
       <c r="B62" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="63">
@@ -1028,7 +1029,7 @@
         </is>
       </c>
       <c r="B63" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="64">
@@ -1038,7 +1039,7 @@
         </is>
       </c>
       <c r="B64" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="65">
@@ -1048,7 +1049,7 @@
         </is>
       </c>
       <c r="B65" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="66">
@@ -1058,7 +1059,7 @@
         </is>
       </c>
       <c r="B66" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="67">
@@ -1068,7 +1069,7 @@
         </is>
       </c>
       <c r="B67" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="68">
@@ -1078,7 +1079,7 @@
         </is>
       </c>
       <c r="B68" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="69">
@@ -1088,7 +1089,7 @@
         </is>
       </c>
       <c r="B69" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="70">
@@ -1098,7 +1099,7 @@
         </is>
       </c>
       <c r="B70" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="71">
@@ -1108,7 +1109,7 @@
         </is>
       </c>
       <c r="B71" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="72">
@@ -1118,7 +1119,7 @@
         </is>
       </c>
       <c r="B72" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="73">
@@ -1128,7 +1129,7 @@
         </is>
       </c>
       <c r="B73" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="74">
@@ -1138,7 +1139,7 @@
         </is>
       </c>
       <c r="B74" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="75">
@@ -1148,7 +1149,7 @@
         </is>
       </c>
       <c r="B75" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="76">
@@ -1158,7 +1159,7 @@
         </is>
       </c>
       <c r="B76" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="77">
@@ -1168,7 +1169,7 @@
         </is>
       </c>
       <c r="B77" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="78">
@@ -1178,7 +1179,7 @@
         </is>
       </c>
       <c r="B78" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="79">
@@ -1188,7 +1189,7 @@
         </is>
       </c>
       <c r="B79" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="80">
@@ -1198,7 +1199,7 @@
         </is>
       </c>
       <c r="B80" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="81">
@@ -1208,7 +1209,7 @@
         </is>
       </c>
       <c r="B81" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="82">
@@ -1218,7 +1219,7 @@
         </is>
       </c>
       <c r="B82" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="83">
@@ -1228,7 +1229,7 @@
         </is>
       </c>
       <c r="B83" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="84">
@@ -1238,7 +1239,7 @@
         </is>
       </c>
       <c r="B84" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="85">
@@ -1248,7 +1249,7 @@
         </is>
       </c>
       <c r="B85" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="86">
@@ -1258,7 +1259,7 @@
         </is>
       </c>
       <c r="B86" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="87">
@@ -1268,7 +1269,7 @@
         </is>
       </c>
       <c r="B87" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="88">
@@ -1278,7 +1279,486 @@
         </is>
       </c>
       <c r="B88" s="1" t="n">
-        <v>46109</v>
+        <v>46110</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="10.08984375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Docket No.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date Last Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>21-0719</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>26-0047</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>25-0945</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>22-0432</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>22-0442</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>25-0611</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>25-0383</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>25-0495</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>24-0813</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>17-0331</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>25-0213</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>23-0068</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>23-0069</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>21-0159</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>24-0680</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>21-0155</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>12-0528</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>24-0460</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>23-0055</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>24-0181</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>22-0486</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>24-0577</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>24-0484</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24-0378</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>24-0676</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>24-0675</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>24-0677</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>24-0674</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>23-0714</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>25-0435</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>23-0622</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>25-0212</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>25-0240</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>24-0727</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>23-0675</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18-1725</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>24-0396</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>24-0279</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>23-0770</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>23-0345</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>22-0749</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>24-0394</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>24-0237</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>23-0665</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>46110</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>22-0499</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>46110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>